<commit_message>
fix: keep a picture's oneCell or absolute two-cell anchor on save (#780)
Excel anchors an inserted picture as xdr:twoCellAnchor editAs="oneCell" and places and sizes every two-cell anchor from its from/to markers. The load kept only the top-left cell and took size and position from a:xfrm, so the save wrote a oneCellAnchor at the xfrm size or an absoluteAnchor at the xfrm offset. A picture whose xfrm held 0,0 and its native size shrank or jumped to the sheet's corner.

The loaded markers are now kept on XLKeptAnchor. An unedited picture is written back by editing its loaded anchor in place (marker cells, name, image link only). Row and column edits move a oneCell anchor by its top-left shift and leave an absolute anchor alone, as Excel does. Any edit of placement, size or position drops the kept anchor.

ImageShapeZOrder-Output.xlsx is regenerated: its picture is an Excel oneCell anchor, which it previously recorded as a converted oneCellAnchor.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Other/Pictures/ImageShapeZOrder-Output.xlsx
+++ b/XLibur.Tests/Resource/Other/Pictures/ImageShapeZOrder-Output.xlsx
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<xdr:wsDr xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
@@ -161,37 +161,56 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5657850" cy="3086100"/>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>169445</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="図 4"/>
+        <xdr:cNvPr id="2" name="図 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{04541A4C-6DF3-ABFB-463C-094A833E30B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="5657850" cy="3086100"/>
+          <a:off x="609600" y="647700"/>
+          <a:ext cx="5655845" cy="3086100"/>
         </a:xfrm>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:oneCellAnchor>
+  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>

</xml_diff>